<commit_message>
Rebuild Seasons at Meridian supply chart with HelloData 5-mi unit details
HD mix-weighted subject rents drive the subject rows; comp lease-up
occupancy/pace from HD cumulative leases (Village ~12%, Wesley ~48%,
Tauri ~100% pre-leased at ~20/mo).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gzof5jycbxc5BFsHyg4DJw
</commit_message>
<xml_diff>
--- a/SeasonsMeridian/supply/Seasons_at_Meridian__Supply_Chart.xlsx
+++ b/SeasonsMeridian/supply/Seasons_at_Meridian__Supply_Chart.xlsx
@@ -1019,7 +1019,7 @@
         <v>0.9879520000000001</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>1664</v>
+        <v>1651.435028248588</v>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
@@ -1189,7 +1189,7 @@
         <v>0.990196</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>1683</v>
+        <v>1665.511627906977</v>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
@@ -1235,7 +1235,7 @@
         <v>1</v>
       </c>
       <c r="G13" s="10" t="n">
-        <v>2110</v>
+        <v>1747.513661202186</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -1250,7 +1250,11 @@
           <t>Garden</t>
         </is>
       </c>
-      <c r="K13" s="7" t="n"/>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>Rent: HD mix-wtd $1,748 vs CoStar ask $2,110</t>
+        </is>
+      </c>
       <c r="M13">
         <f>IFERROR(VALUE(RIGHT(E13,4))*4+MATCH(LEFT(E13,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
@@ -1277,7 +1281,7 @@
         <v>0.989011</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>1189</v>
+        <v>1165.555555555556</v>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
@@ -1363,7 +1367,7 @@
         <v>0.948148</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>2229</v>
+        <v>2164.319806763285</v>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
@@ -1493,7 +1497,7 @@
         <v>0.945833</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>1689</v>
+        <v>1624.407772304324</v>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
@@ -1585,7 +1589,7 @@
         <v>0.763889</v>
       </c>
       <c r="G21" s="10" t="n">
-        <v>1707</v>
+        <v>1735.469387755102</v>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
@@ -1631,7 +1635,7 @@
         <v>0.990196</v>
       </c>
       <c r="G22" s="10" t="n">
-        <v>1898</v>
+        <v>1884.446808510638</v>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
@@ -1673,7 +1677,7 @@
         <v>0.933333</v>
       </c>
       <c r="G23" s="10" t="n">
-        <v>2070</v>
+        <v>1995</v>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
@@ -1715,7 +1719,7 @@
         <v>1</v>
       </c>
       <c r="G24" s="10" t="n">
-        <v>2595</v>
+        <v>2489.375</v>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
@@ -1757,7 +1761,7 @@
         <v>0.969697</v>
       </c>
       <c r="G25" s="10" t="n">
-        <v>1762</v>
+        <v>1739.209026472431</v>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
@@ -1850,10 +1854,10 @@
         </is>
       </c>
       <c r="F29" s="17" t="n">
-        <v>0.803571</v>
+        <v>0.119047619047619</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>1742</v>
+        <v>1747.513661202186</v>
       </c>
       <c r="H29" s="15" t="inlineStr">
         <is>
@@ -1870,7 +1874,7 @@
       </c>
       <c r="K29" s="15" t="inlineStr">
         <is>
-          <t>Units: CoStar 336 vs RealPage 96; Year built: 2018/2024; Units: CoStar 336 vs RealPage 36; Year built: 2021/2024; Units: CoStar 336 vs RealPage 64; Year built: 1993/2024; Units: CoStar 336 vs RealPage 336; Year built: 2024/2027; Occ: CoStar 80% vs RealPage 11%; Verify rent/occ w/ HelloData</t>
+          <t>Units: CoStar 336 vs RealPage 96; Year built: 2018/2024; Units: CoStar 336 vs RealPage 36; Year built: 2021/2024; Units: CoStar 336 vs RealPage 64; Year built: 1993/2024; Units: CoStar 336 vs RealPage 336; Year built: 2024/2027; Occ: CoStar 80% vs RealPage 11%; Occ: HD ~12% (CoStar/RP showed 80%); HD (90d): occ ~12% (units leased), ~13 leases/mo</t>
         </is>
       </c>
       <c r="M29">
@@ -1896,10 +1900,10 @@
         </is>
       </c>
       <c r="F30" s="17" t="n">
-        <v>0.277487</v>
+        <v>0.4764397905759162</v>
       </c>
       <c r="G30" s="18" t="n">
-        <v>1716</v>
+        <v>1994.484728234728</v>
       </c>
       <c r="H30" s="15" t="inlineStr">
         <is>
@@ -1916,7 +1920,7 @@
       </c>
       <c r="K30" s="15" t="inlineStr">
         <is>
-          <t>Occ: CoStar 28% vs RealPage 84%; Rent: CoStar ask $1,716 vs RealPage eff $2,004; Verify rent/occ w/ HelloData</t>
+          <t>Occ: CoStar 28% vs RealPage 84%; Rent: CoStar ask $1,716 vs RealPage eff $2,004; Rent: HD mix-wtd $1,994 vs CoStar ask $1,716; Occ: HD ~48% (CoStar/RP showed 28%); HD (90d): occ ~48% (units leased), ~22 leases/mo</t>
         </is>
       </c>
       <c r="M30">
@@ -1990,10 +1994,10 @@
         </is>
       </c>
       <c r="F32" s="17" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="G32" s="18" t="n">
-        <v>1862</v>
+        <v>1833.726076373041</v>
       </c>
       <c r="H32" s="15" t="inlineStr">
         <is>
@@ -2010,7 +2014,7 @@
       </c>
       <c r="K32" s="15" t="inlineStr">
         <is>
-          <t>Units: CoStar 156 vs RealPage 128; Year built: 2026/2027; Occ: CoStar 25% vs RealPage 18%; Rent: CoStar ask $1,862 vs RealPage eff $1,684; Verify rent/occ w/ HelloData</t>
+          <t>Units: CoStar 156 vs RealPage 128; Year built: 2026/2027; Occ: CoStar 25% vs RealPage 18%; Rent: CoStar ask $1,862 vs RealPage eff $1,684; Occ: HD ~100% (CoStar/RP showed 25%); HD (90d): occ ~100% (units leased), ~20 leases/mo</t>
         </is>
       </c>
       <c r="M32">
@@ -2939,7 +2943,7 @@
     <row r="59">
       <c r="B59" s="36" t="inlineStr">
         <is>
-          <t>* 5-Mile radius. Rent ($) = market asking. Proximity (mi) = straight-line distance from the subject. Est. Delivery drives the Supply &amp; Absorption tab's per-window supply (edit it there or here — they are linked). See the 'Supply &amp; Absorption' tab for the forward supply / absorption / overall-occupancy forecast.</t>
+          <t>* 5-Mile radius. Rent ($) = HelloData mix-weighted asking where covered, else market asking (CoStar). Proximity (mi) = straight-line distance from the subject. Est. Delivery drives the Supply &amp; Absorption tab's per-window supply (edit it there or here — they are linked). See the 'Supply &amp; Absorption' tab for the forward supply / absorption / overall-occupancy forecast.</t>
         </is>
       </c>
     </row>
@@ -3891,10 +3895,10 @@
         <v>1835</v>
       </c>
       <c r="H23" s="56" t="n">
-        <v>1801</v>
+        <v>1777</v>
       </c>
       <c r="I23" s="56">
-        <f>IFERROR('Cash Flow (Annual)'!$F$4,1868)</f>
+        <f>IFERROR('Cash Flow (Annual)'!$F$4,1735)</f>
         <v/>
       </c>
       <c r="J23" s="57">
@@ -4052,10 +4056,10 @@
         <v>1835</v>
       </c>
       <c r="H25" s="56" t="n">
-        <v>1669</v>
+        <v>1619</v>
       </c>
       <c r="I25" s="56">
-        <f>IFERROR('Cash Flow (Annual)'!$F$5,1689)</f>
+        <f>IFERROR('Cash Flow (Annual)'!$F$5,1578)</f>
         <v/>
       </c>
       <c r="J25" s="57">
@@ -5211,7 +5215,7 @@
       </c>
       <c r="E66" s="79" t="inlineStr">
         <is>
-          <t>CoStar</t>
+          <t>HD</t>
         </is>
       </c>
     </row>
@@ -5223,7 +5227,7 @@
       </c>
       <c r="E67" s="79" t="inlineStr">
         <is>
-          <t>HD occ + CoStar rents</t>
+          <t>HD</t>
         </is>
       </c>
     </row>
@@ -5510,8 +5514,12 @@
       <c r="L3" s="82" t="n">
         <v>1841</v>
       </c>
-      <c r="M3" s="82" t="n"/>
-      <c r="N3" s="82" t="n"/>
+      <c r="M3" s="82" t="n">
+        <v>1739.209026472431</v>
+      </c>
+      <c r="N3" s="82" t="n">
+        <v>1663.812235275689</v>
+      </c>
       <c r="O3" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -5564,8 +5572,12 @@
         <v>2595</v>
       </c>
       <c r="L4" s="82" t="n"/>
-      <c r="M4" s="82" t="n"/>
-      <c r="N4" s="82" t="n"/>
+      <c r="M4" s="82" t="n">
+        <v>2489.375</v>
+      </c>
+      <c r="N4" s="82" t="n">
+        <v>2395.895833333333</v>
+      </c>
       <c r="O4" t="inlineStr">
         <is>
           <t>CoStar</t>
@@ -5614,8 +5626,12 @@
         <v>2070</v>
       </c>
       <c r="L5" s="82" t="n"/>
-      <c r="M5" s="82" t="n"/>
-      <c r="N5" s="82" t="n"/>
+      <c r="M5" s="82" t="n">
+        <v>1995</v>
+      </c>
+      <c r="N5" s="82" t="n">
+        <v>1995</v>
+      </c>
       <c r="O5" t="inlineStr">
         <is>
           <t>CoStar</t>
@@ -5664,8 +5680,12 @@
         <v>1898</v>
       </c>
       <c r="L6" s="82" t="n"/>
-      <c r="M6" s="82" t="n"/>
-      <c r="N6" s="82" t="n"/>
+      <c r="M6" s="82" t="n">
+        <v>1884.446808510638</v>
+      </c>
+      <c r="N6" s="82" t="n">
+        <v>1884.446808510638</v>
+      </c>
       <c r="O6" t="inlineStr">
         <is>
           <t>CoStar</t>
@@ -5718,8 +5738,12 @@
       <c r="L7" s="82" t="n">
         <v>1754</v>
       </c>
-      <c r="M7" s="82" t="n"/>
-      <c r="N7" s="82" t="n"/>
+      <c r="M7" s="82" t="n">
+        <v>1624.407772304324</v>
+      </c>
+      <c r="N7" s="82" t="n">
+        <v>1573.192255062945</v>
+      </c>
       <c r="O7" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -5834,8 +5858,12 @@
       <c r="L9" s="82" t="n">
         <v>1691</v>
       </c>
-      <c r="M9" s="82" t="n"/>
-      <c r="N9" s="82" t="n"/>
+      <c r="M9" s="82" t="n">
+        <v>1735.469387755102</v>
+      </c>
+      <c r="N9" s="82" t="n">
+        <v>1735.469387755102</v>
+      </c>
       <c r="O9" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -5942,8 +5970,12 @@
       <c r="L11" s="82" t="n">
         <v>2243</v>
       </c>
-      <c r="M11" s="82" t="n"/>
-      <c r="N11" s="82" t="n"/>
+      <c r="M11" s="82" t="n">
+        <v>2164.319806763285</v>
+      </c>
+      <c r="N11" s="82" t="n">
+        <v>2140.342028985508</v>
+      </c>
       <c r="O11" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -6046,8 +6078,12 @@
         <v>1189</v>
       </c>
       <c r="L13" s="82" t="n"/>
-      <c r="M13" s="82" t="n"/>
-      <c r="N13" s="82" t="n"/>
+      <c r="M13" s="82" t="n">
+        <v>1165.555555555556</v>
+      </c>
+      <c r="N13" s="82" t="n">
+        <v>1156.326599326599</v>
+      </c>
       <c r="O13" t="inlineStr">
         <is>
           <t>CoStar</t>
@@ -6146,8 +6182,12 @@
       <c r="L15" s="82" t="n">
         <v>1661</v>
       </c>
-      <c r="M15" s="82" t="n"/>
-      <c r="N15" s="82" t="n"/>
+      <c r="M15" s="82" t="n">
+        <v>1665.511627906977</v>
+      </c>
+      <c r="N15" s="82" t="n">
+        <v>1665.511627906977</v>
+      </c>
       <c r="O15" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -6198,14 +6238,22 @@
         <v>2110</v>
       </c>
       <c r="L16" s="82" t="n"/>
-      <c r="M16" s="82" t="n"/>
-      <c r="N16" s="82" t="n"/>
+      <c r="M16" s="82" t="n">
+        <v>1747.513661202186</v>
+      </c>
+      <c r="N16" s="82" t="n">
+        <v>1747.513661202186</v>
+      </c>
       <c r="O16" t="inlineStr">
         <is>
           <t>CoStar</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Rent: HD mix-wtd $1,748 vs CoStar ask $2,110</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6252,8 +6300,12 @@
       <c r="L17" s="82" t="n">
         <v>1641</v>
       </c>
-      <c r="M17" s="82" t="n"/>
-      <c r="N17" s="82" t="n"/>
+      <c r="M17" s="82" t="n">
+        <v>1651.435028248588</v>
+      </c>
+      <c r="N17" s="82" t="n">
+        <v>1651.435028248588</v>
+      </c>
       <c r="O17" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -6542,15 +6594,21 @@
       <c r="I23" s="81" t="n">
         <v>0.18</v>
       </c>
-      <c r="J23" s="81" t="n"/>
+      <c r="J23" s="81" t="n">
+        <v>1</v>
+      </c>
       <c r="K23" s="82" t="n">
         <v>1862</v>
       </c>
       <c r="L23" s="82" t="n">
         <v>1684</v>
       </c>
-      <c r="M23" s="82" t="n"/>
-      <c r="N23" s="82" t="n"/>
+      <c r="M23" s="82" t="n">
+        <v>1833.726076373041</v>
+      </c>
+      <c r="N23" s="82" t="n">
+        <v>1813.154621177544</v>
+      </c>
       <c r="O23" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -6558,7 +6616,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Units: CoStar 156 vs RealPage 128; Year built: 2026/2027; Occ: CoStar 25% vs RealPage 18%; Rent: CoStar ask $1,862 vs RealPage eff $1,684; Verify rent/occ w/ HelloData</t>
+          <t>Units: CoStar 156 vs RealPage 128; Year built: 2026/2027; Occ: CoStar 25% vs RealPage 18%; Rent: CoStar ask $1,862 vs RealPage eff $1,684; Occ: HD ~100% (CoStar/RP showed 25%); HD (90d): occ ~100% (units leased), ~20 leases/mo</t>
         </is>
       </c>
     </row>
@@ -6701,15 +6759,21 @@
       <c r="I26" s="81" t="n">
         <v>0.113</v>
       </c>
-      <c r="J26" s="81" t="n"/>
+      <c r="J26" s="81" t="n">
+        <v>0.119047619047619</v>
+      </c>
       <c r="K26" s="82" t="n">
         <v>1742</v>
       </c>
       <c r="L26" s="82" t="n">
         <v>1677</v>
       </c>
-      <c r="M26" s="82" t="n"/>
-      <c r="N26" s="82" t="n"/>
+      <c r="M26" s="82" t="n">
+        <v>1747.513661202186</v>
+      </c>
+      <c r="N26" s="82" t="n">
+        <v>1747.513661202186</v>
+      </c>
       <c r="O26" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -6717,7 +6781,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>Units: CoStar 336 vs RealPage 96; Year built: 2018/2024; Units: CoStar 336 vs RealPage 36; Year built: 2021/2024; Units: CoStar 336 vs RealPage 64; Year built: 1993/2024; Units: CoStar 336 vs RealPage 336; Year built: 2024/2027; Occ: CoStar 80% vs RealPage 11%; Verify rent/occ w/ HelloData</t>
+          <t>Units: CoStar 336 vs RealPage 96; Year built: 2018/2024; Units: CoStar 336 vs RealPage 36; Year built: 2021/2024; Units: CoStar 336 vs RealPage 64; Year built: 1993/2024; Units: CoStar 336 vs RealPage 336; Year built: 2024/2027; Occ: CoStar 80% vs RealPage 11%; Occ: HD ~12% (CoStar/RP showed 80%); HD (90d): occ ~12% (units leased), ~13 leases/mo</t>
         </is>
       </c>
     </row>
@@ -6759,15 +6823,21 @@
       <c r="I27" s="81" t="n">
         <v>0.838</v>
       </c>
-      <c r="J27" s="81" t="n"/>
+      <c r="J27" s="81" t="n">
+        <v>0.4764397905759162</v>
+      </c>
       <c r="K27" s="82" t="n">
         <v>1716</v>
       </c>
       <c r="L27" s="82" t="n">
         <v>2004</v>
       </c>
-      <c r="M27" s="82" t="n"/>
-      <c r="N27" s="82" t="n"/>
+      <c r="M27" s="82" t="n">
+        <v>1994.484728234728</v>
+      </c>
+      <c r="N27" s="82" t="n">
+        <v>1994.484728234728</v>
+      </c>
       <c r="O27" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -6775,7 +6845,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>Occ: CoStar 28% vs RealPage 84%; Rent: CoStar ask $1,716 vs RealPage eff $2,004; Verify rent/occ w/ HelloData</t>
+          <t>Occ: CoStar 28% vs RealPage 84%; Rent: CoStar ask $1,716 vs RealPage eff $2,004; Rent: HD mix-wtd $1,994 vs CoStar ask $1,716; Occ: HD ~48% (CoStar/RP showed 28%); HD (90d): occ ~48% (units leased), ~22 leases/mo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add The Judy (Hawkins, 162u at Maple Grove & Overland) to Seasons supply chart from OM
- apply_diligence() can now CREATE a deal from an unmatched pipeline row
  (analyst-sourced: an OM, permit, or planning file) with units, status,
  est_delivery and exact coordinates — vendor-untracked deals chart like
  any other comp.
- The Judy: 162u Class A garden, 1770 S Maple Grove Rd (3.4 mi from
  Seasons), construction targeted Q3 2026, est first units Q1 2028; not in
  CoStar or RealPage. Land-use site 177 had the parcel as developable
  vacant at Medium MF-threat (R-2 conditional) — OM proves the conditional
  path exercised; crosswalk reclassifies it latent -> tracked pipeline.
- OM saved to research/oms/; chart, maps, viewers, crosswalk refreshed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gzof5jycbxc5BFsHyg4DJw
</commit_message>
<xml_diff>
--- a/SeasonsMeridian/supply/Seasons_at_Meridian__Supply_Chart.xlsx
+++ b/SeasonsMeridian/supply/Seasons_at_Meridian__Supply_Chart.xlsx
@@ -815,7 +815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:M54"/>
+  <dimension ref="B2:M55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2166,7 +2166,7 @@
       <c r="B39" s="28" t="n"/>
       <c r="C39" s="29" t="inlineStr">
         <is>
-          <t>PROPOSED (12 properties, 3,014 units)</t>
+          <t>PROPOSED (13 properties, 3,176 units)</t>
         </is>
       </c>
     </row>
@@ -2222,15 +2222,15 @@
       </c>
       <c r="C41" s="31" t="inlineStr">
         <is>
-          <t>Victory Flats</t>
+          <t>The Judy (Maple Grove &amp; Overland)</t>
         </is>
       </c>
       <c r="D41" s="32" t="n">
-        <v>301</v>
+        <v>162</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
-          <t>Q3 2028</t>
+          <t>Q1 2028</t>
         </is>
       </c>
       <c r="F41" s="33" t="n"/>
@@ -2241,20 +2241,16 @@
       </c>
       <c r="H41" s="31" t="inlineStr">
         <is>
-          <t>Welltower Inc.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" s="35" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="J41" s="30" t="inlineStr">
-        <is>
-          <t>Townhome</t>
-        </is>
-      </c>
+        <v>3.4</v>
+      </c>
+      <c r="J41" s="30" t="n"/>
       <c r="K41" s="31" t="inlineStr">
         <is>
-          <t>Diligence: proposed</t>
+          <t>Analyst-sourced deal (not in CoStar/RealPage); Diligence: proposed - equity raise underway; construction targeted Q3 2026</t>
         </is>
       </c>
       <c r="M41">
@@ -2268,15 +2264,15 @@
       </c>
       <c r="C42" s="31" t="inlineStr">
         <is>
-          <t>The Gateway at Ten Mile</t>
+          <t>Victory Flats</t>
         </is>
       </c>
       <c r="D42" s="32" t="n">
-        <v>390</v>
+        <v>301</v>
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Q4 2028</t>
+          <t>Q3 2028</t>
         </is>
       </c>
       <c r="F42" s="33" t="n"/>
@@ -2287,15 +2283,15 @@
       </c>
       <c r="H42" s="31" t="inlineStr">
         <is>
-          <t>TGI Corp</t>
+          <t>Welltower Inc.</t>
         </is>
       </c>
       <c r="I42" s="35" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="J42" s="30" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Townhome</t>
         </is>
       </c>
       <c r="K42" s="31" t="inlineStr">
@@ -2314,15 +2310,15 @@
       </c>
       <c r="C43" s="31" t="inlineStr">
         <is>
-          <t>Ascent Overland</t>
+          <t>The Gateway at Ten Mile</t>
         </is>
       </c>
       <c r="D43" s="32" t="n">
-        <v>138</v>
+        <v>390</v>
       </c>
       <c r="E43" s="30" t="inlineStr">
         <is>
-          <t>Q1 2029</t>
+          <t>Q4 2028</t>
         </is>
       </c>
       <c r="F43" s="33" t="n"/>
@@ -2333,11 +2329,11 @@
       </c>
       <c r="H43" s="31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TGI Corp</t>
         </is>
       </c>
       <c r="I43" s="35" t="n">
-        <v>1.5</v>
+        <v>3.7</v>
       </c>
       <c r="J43" s="30" t="inlineStr">
         <is>
@@ -2360,15 +2356,15 @@
       </c>
       <c r="C44" s="31" t="inlineStr">
         <is>
-          <t>Record</t>
+          <t>Ascent Overland</t>
         </is>
       </c>
       <c r="D44" s="32" t="n">
-        <v>472</v>
+        <v>138</v>
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Q1 2029</t>
         </is>
       </c>
       <c r="F44" s="33" t="n"/>
@@ -2383,7 +2379,7 @@
         </is>
       </c>
       <c r="I44" s="35" t="n">
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="J44" s="30" t="inlineStr">
         <is>
@@ -2392,7 +2388,7 @@
       </c>
       <c r="K44" s="31" t="inlineStr">
         <is>
-          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
+          <t>Diligence: proposed</t>
         </is>
       </c>
       <c r="M44">
@@ -2406,11 +2402,11 @@
       </c>
       <c r="C45" s="31" t="inlineStr">
         <is>
-          <t>Syringa Crossing</t>
+          <t>Record</t>
         </is>
       </c>
       <c r="D45" s="32" t="n">
-        <v>322</v>
+        <v>472</v>
       </c>
       <c r="E45" s="30" t="inlineStr">
         <is>
@@ -2429,7 +2425,7 @@
         </is>
       </c>
       <c r="I45" s="35" t="n">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
       <c r="J45" s="30" t="inlineStr">
         <is>
@@ -2452,11 +2448,11 @@
       </c>
       <c r="C46" s="31" t="inlineStr">
         <is>
-          <t>12565 West Fairview Avenue</t>
+          <t>Syringa Crossing</t>
         </is>
       </c>
       <c r="D46" s="32" t="n">
-        <v>275</v>
+        <v>322</v>
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
@@ -2475,7 +2471,7 @@
         </is>
       </c>
       <c r="I46" s="35" t="n">
-        <v>2.1</v>
+        <v>2.8</v>
       </c>
       <c r="J46" s="30" t="inlineStr">
         <is>
@@ -2498,11 +2494,11 @@
       </c>
       <c r="C47" s="31" t="inlineStr">
         <is>
-          <t>Cobalt Point</t>
+          <t>12565 West Fairview Avenue</t>
         </is>
       </c>
       <c r="D47" s="32" t="n">
-        <v>264</v>
+        <v>275</v>
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
@@ -2521,11 +2517,11 @@
         </is>
       </c>
       <c r="I47" s="35" t="n">
-        <v>0.6</v>
+        <v>2.1</v>
       </c>
       <c r="J47" s="30" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K47" s="31" t="inlineStr">
@@ -2544,11 +2540,11 @@
       </c>
       <c r="C48" s="31" t="inlineStr">
         <is>
-          <t>12548 West Overland Road</t>
+          <t>Cobalt Point</t>
         </is>
       </c>
       <c r="D48" s="32" t="n">
-        <v>156</v>
+        <v>264</v>
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
@@ -2567,11 +2563,11 @@
         </is>
       </c>
       <c r="I48" s="35" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="J48" s="30" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K48" s="31" t="inlineStr">
@@ -2590,11 +2586,11 @@
       </c>
       <c r="C49" s="31" t="inlineStr">
         <is>
-          <t>Fairview</t>
+          <t>12548 West Overland Road</t>
         </is>
       </c>
       <c r="D49" s="32" t="n">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="E49" s="30" t="inlineStr">
         <is>
@@ -2613,11 +2609,11 @@
         </is>
       </c>
       <c r="I49" s="35" t="n">
-        <v>2.1</v>
+        <v>1.1</v>
       </c>
       <c r="J49" s="30" t="inlineStr">
         <is>
-          <t>Townhome</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K49" s="31" t="inlineStr">
@@ -2636,11 +2632,11 @@
       </c>
       <c r="C50" s="31" t="inlineStr">
         <is>
-          <t>The Cole Denton</t>
+          <t>Fairview</t>
         </is>
       </c>
       <c r="D50" s="32" t="n">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
@@ -2659,11 +2655,11 @@
         </is>
       </c>
       <c r="I50" s="35" t="n">
-        <v>4.5</v>
+        <v>2.1</v>
       </c>
       <c r="J50" s="30" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Townhome</t>
         </is>
       </c>
       <c r="K50" s="31" t="inlineStr">
@@ -2682,11 +2678,11 @@
       </c>
       <c r="C51" s="31" t="inlineStr">
         <is>
-          <t>Meridian OZ Apartments</t>
+          <t>The Cole Denton</t>
         </is>
       </c>
       <c r="D51" s="32" t="n">
-        <v>60</v>
+        <v>136</v>
       </c>
       <c r="E51" s="30" t="inlineStr">
         <is>
@@ -2701,20 +2697,20 @@
       </c>
       <c r="H51" s="31" t="inlineStr">
         <is>
-          <t>Peak Capital Investments Llc</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I51" s="35" t="n">
-        <v>1.1</v>
+        <v>4.5</v>
       </c>
       <c r="J51" s="30" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K51" s="31" t="inlineStr">
         <is>
-          <t>Diligence: proposed</t>
+          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
       </c>
       <c r="M51">
@@ -2722,8 +2718,54 @@
         <v/>
       </c>
     </row>
-    <row r="54">
-      <c r="B54" s="36" t="inlineStr">
+    <row r="52">
+      <c r="B52" s="30" t="n">
+        <v>41</v>
+      </c>
+      <c r="C52" s="31" t="inlineStr">
+        <is>
+          <t>Meridian OZ Apartments</t>
+        </is>
+      </c>
+      <c r="D52" s="32" t="n">
+        <v>60</v>
+      </c>
+      <c r="E52" s="30" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F52" s="33" t="n"/>
+      <c r="G52" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H52" s="31" t="inlineStr">
+        <is>
+          <t>Peak Capital Investments Llc</t>
+        </is>
+      </c>
+      <c r="I52" s="35" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J52" s="30" t="inlineStr">
+        <is>
+          <t>Garden</t>
+        </is>
+      </c>
+      <c r="K52" s="31" t="inlineStr">
+        <is>
+          <t>Diligence: proposed</t>
+        </is>
+      </c>
+      <c r="M52">
+        <f>IFERROR(VALUE(RIGHT(E52,4))*4+MATCH(LEFT(E52,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="36" t="inlineStr">
         <is>
           <t>* 5-Mile radius. Rent ($) = HelloData mix-weighted asking where covered, else market asking (CoStar). Proximity (mi) = straight-line distance from the subject. Est. Delivery drives the Supply &amp; Absorption tab's per-window supply (edit it there or here — they are linked). See the 'Supply &amp; Absorption' tab for the forward supply / absorption / overall-occupancy forecast.</t>
         </is>
@@ -2735,8 +2777,8 @@
     <mergeCell ref="C5:K5"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="C28:K28"/>
+    <mergeCell ref="B55:K55"/>
     <mergeCell ref="C39:K39"/>
-    <mergeCell ref="B54:K54"/>
     <mergeCell ref="C35:K35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3264,13 +3306,17 @@
       </c>
       <c r="R17" s="43" t="inlineStr">
         <is>
-          <t>12548 West Overland Road</t>
+          <t>The Judy (Maple Grove &amp; Overland)</t>
         </is>
       </c>
       <c r="S17" s="44" t="n">
-        <v>156</v>
-      </c>
-      <c r="T17" s="48" t="inlineStr"/>
+        <v>162</v>
+      </c>
+      <c r="T17" s="48" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
       <c r="U17" s="48" t="inlineStr">
         <is>
           <t>Bear only</t>
@@ -3351,11 +3397,11 @@
       </c>
       <c r="R18" s="43" t="inlineStr">
         <is>
-          <t>Fairview</t>
+          <t>12548 West Overland Road</t>
         </is>
       </c>
       <c r="S18" s="44" t="n">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="T18" s="48" t="inlineStr"/>
       <c r="U18" s="48" t="inlineStr">
@@ -3401,46 +3447,42 @@
         <v>450</v>
       </c>
       <c r="I19" s="52">
-        <f>SUMIFS('Competitive Analysis'!$D$5:$D$51,'Competitive Analysis'!$M$5:$M$51,"&gt;="&amp;8102,'Competitive Analysis'!$M$5:$M$51,"&lt;="&amp;8105)</f>
+        <f>SUMIFS('Competitive Analysis'!$D$5:$D$52,'Competitive Analysis'!$M$5:$M$52,"&gt;="&amp;8102,'Competitive Analysis'!$M$5:$M$52,"&lt;="&amp;8105)</f>
         <v/>
       </c>
       <c r="J19" s="53">
-        <f>SUMIFS($S$5:$S$6,$W$5:$W$6,1)+SUMIFS($S$10:$S$21,$W$10:$W$21,1,$X$10:$X$21,1)</f>
+        <f>SUMIFS($S$5:$S$6,$W$5:$W$6,1)+SUMIFS($S$10:$S$22,$W$10:$W$22,1,$X$10:$X$22,1)</f>
         <v/>
       </c>
       <c r="K19" s="53">
-        <f>SUMIFS($S$5:$S$6,$W$5:$W$6,2)+SUMIFS($S$10:$S$21,$W$10:$W$21,2,$X$10:$X$21,1)</f>
+        <f>SUMIFS($S$5:$S$6,$W$5:$W$6,2)+SUMIFS($S$10:$S$22,$W$10:$W$22,2,$X$10:$X$22,1)</f>
         <v/>
       </c>
       <c r="L19" s="53">
-        <f>SUMIFS($S$5:$S$6,$W$5:$W$6,3)+SUMIFS($S$10:$S$21,$W$10:$W$21,3,$X$10:$X$21,1)</f>
+        <f>SUMIFS($S$5:$S$6,$W$5:$W$6,3)+SUMIFS($S$10:$S$22,$W$10:$W$22,3,$X$10:$X$22,1)</f>
         <v/>
       </c>
       <c r="M19" s="53">
-        <f>SUMIFS($S$5:$S$6,$W$5:$W$6,4)+SUMIFS($S$10:$S$21,$W$10:$W$21,4,$X$10:$X$21,1)</f>
+        <f>SUMIFS($S$5:$S$6,$W$5:$W$6,4)+SUMIFS($S$10:$S$22,$W$10:$W$22,4,$X$10:$X$22,1)</f>
         <v/>
       </c>
       <c r="N19" s="53">
-        <f>SUMIFS($S$5:$S$6,$W$5:$W$6,5)+SUMIFS($S$10:$S$21,$W$10:$W$21,5,$X$10:$X$21,1)</f>
+        <f>SUMIFS($S$5:$S$6,$W$5:$W$6,5)+SUMIFS($S$10:$S$22,$W$10:$W$22,5,$X$10:$X$22,1)</f>
         <v/>
       </c>
       <c r="O19" s="53">
-        <f>SUMIFS($S$5:$S$6,$W$5:$W$6,6)+SUMIFS($S$10:$S$21,$W$10:$W$21,6,$X$10:$X$21,1)</f>
+        <f>SUMIFS($S$5:$S$6,$W$5:$W$6,6)+SUMIFS($S$10:$S$22,$W$10:$W$22,6,$X$10:$X$22,1)</f>
         <v/>
       </c>
       <c r="R19" s="43" t="inlineStr">
         <is>
-          <t>Ascent Overland</t>
+          <t>Fairview</t>
         </is>
       </c>
       <c r="S19" s="44" t="n">
-        <v>138</v>
-      </c>
-      <c r="T19" s="48" t="inlineStr">
-        <is>
-          <t>Q1 2029</t>
-        </is>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="T19" s="48" t="inlineStr"/>
       <c r="U19" s="48" t="inlineStr">
         <is>
           <t>Bear only</t>
@@ -3512,13 +3554,17 @@
       </c>
       <c r="R20" s="43" t="inlineStr">
         <is>
-          <t>The Cole Denton</t>
+          <t>Ascent Overland</t>
         </is>
       </c>
       <c r="S20" s="44" t="n">
-        <v>136</v>
-      </c>
-      <c r="T20" s="48" t="inlineStr"/>
+        <v>138</v>
+      </c>
+      <c r="T20" s="48" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
       <c r="U20" s="48" t="inlineStr">
         <is>
           <t>Bear only</t>
@@ -3591,11 +3637,11 @@
       </c>
       <c r="R21" s="43" t="inlineStr">
         <is>
-          <t>Meridian OZ Apartments</t>
+          <t>The Cole Denton</t>
         </is>
       </c>
       <c r="S21" s="44" t="n">
-        <v>60</v>
+        <v>136</v>
       </c>
       <c r="T21" s="48" t="inlineStr"/>
       <c r="U21" s="48" t="inlineStr">
@@ -3621,6 +3667,32 @@
         <is>
           <t>SUBJECT (Seasons at Meridian)</t>
         </is>
+      </c>
+      <c r="R22" s="43" t="inlineStr">
+        <is>
+          <t>Meridian OZ Apartments</t>
+        </is>
+      </c>
+      <c r="S22" s="44" t="n">
+        <v>60</v>
+      </c>
+      <c r="T22" s="48" t="inlineStr"/>
+      <c r="U22" s="48" t="inlineStr">
+        <is>
+          <t>Bear only</t>
+        </is>
+      </c>
+      <c r="V22">
+        <f>IFERROR(VALUE(RIGHT(T22,4))*4+MATCH(LEFT(T22,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
+      </c>
+      <c r="W22">
+        <f>IF(V22="","",IF(V22&lt;=$Z$1,0,MAX(1,INT((V22-$Z$2)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X22">
+        <f>IF(U22="All",1,IF(U22="Bear+Base",IF($Z$3&gt;=2,1,0),IF(U22="Bear only",IF($Z$3&gt;=3,1,0),0)))</f>
+        <v/>
       </c>
     </row>
     <row r="23" ht="14.4" customHeight="1">
@@ -4948,7 +5020,7 @@
     <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Bear,Base,Bull"</formula1>
     </dataValidation>
-    <dataValidation sqref="U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Bear only,Bear+Base,All,None"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4962,7 +5034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P41"/>
+  <dimension ref="A1:P42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6719,23 +6791,20 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Union 93</t>
+          <t>The Judy (Maple Grove &amp; Overland)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>221-225 E Broadway Ave</t>
+          <t>1770 S Maple Grove Rd, Boise 83704</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>350</v>
-      </c>
-      <c r="D33" t="n">
-        <v>2026</v>
+        <v>162</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Q3 2026</t>
+          <t>Q1 2028</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -6752,28 +6821,36 @@
       <c r="N33" s="82" t="n"/>
       <c r="O33" t="inlineStr">
         <is>
-          <t>CoStar+RealPage</t>
+          <t>Diligence</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>Diligence: stalled - foreclosure since Nov 2022; no restart as of Jul 2026</t>
+          <t>Analyst-sourced deal (not in CoStar/RealPage); Diligence: proposed - equity raise underway; construction targeted Q3 2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Meridian OZ Apartments</t>
+          <t>Union 93</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1475 E Franklin Rd</t>
+          <t>221-225 E Broadway Ave</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>60</v>
+        <v>350</v>
+      </c>
+      <c r="D34" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -6794,23 +6871,23 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Diligence: proposed</t>
+          <t>Diligence: stalled - foreclosure since Nov 2022; no restart as of Jul 2026</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>The Cole Denton</t>
+          <t>Meridian OZ Apartments</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>580 N Cole Rd</t>
+          <t>1475 E Franklin Rd</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>136</v>
+        <v>60</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -6826,28 +6903,28 @@
       <c r="N35" s="82" t="n"/>
       <c r="O35" t="inlineStr">
         <is>
-          <t>RealPage</t>
+          <t>CoStar+RealPage</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
+          <t>Diligence: proposed</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Record</t>
+          <t>The Cole Denton</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>E Fairview Ave &amp; N Records Way</t>
+          <t>580 N Cole Rd</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>472</v>
+        <v>136</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -6875,16 +6952,16 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cobalt Point</t>
+          <t>Record</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>S Cobalt Point Way &amp; E Copper Point Dr</t>
+          <t>E Fairview Ave &amp; N Records Way</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>264</v>
+        <v>472</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -6912,16 +6989,16 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Fairview</t>
+          <t>Cobalt Point</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1005 E Fairview Ave</t>
+          <t>S Cobalt Point Way &amp; E Copper Point Dr</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>150</v>
+        <v>264</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -6933,12 +7010,8 @@
       <c r="J38" s="81" t="n"/>
       <c r="K38" s="82" t="n"/>
       <c r="L38" s="82" t="n"/>
-      <c r="M38" s="82" t="n">
-        <v>1837.580964685616</v>
-      </c>
-      <c r="N38" s="82" t="n">
-        <v>1837.580964685616</v>
-      </c>
+      <c r="M38" s="82" t="n"/>
+      <c r="N38" s="82" t="n"/>
       <c r="O38" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -6953,16 +7026,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>12548 West Overland Road</t>
+          <t>Fairview</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>12548 W Overland Rd</t>
+          <t>1005 E Fairview Ave</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -6974,8 +7047,12 @@
       <c r="J39" s="81" t="n"/>
       <c r="K39" s="82" t="n"/>
       <c r="L39" s="82" t="n"/>
-      <c r="M39" s="82" t="n"/>
-      <c r="N39" s="82" t="n"/>
+      <c r="M39" s="82" t="n">
+        <v>1837.580964685616</v>
+      </c>
+      <c r="N39" s="82" t="n">
+        <v>1837.580964685616</v>
+      </c>
       <c r="O39" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -6990,16 +7067,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>12565 West Fairview Avenue</t>
+          <t>12548 West Overland Road</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>12565 W Fairview Ave</t>
+          <t>12548 W Overland Rd</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>275</v>
+        <v>156</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -7027,16 +7104,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Syringa Crossing</t>
+          <t>12565 West Fairview Avenue</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Amity Ave &amp; Meridian Rd</t>
+          <t>12565 W Fairview Ave</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>322</v>
+        <v>275</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -7056,6 +7133,43 @@
         </is>
       </c>
       <c r="P41" t="inlineStr">
+        <is>
+          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Syringa Crossing</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Amity Ave &amp; Meridian Rd</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>322</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+      <c r="H42" s="81" t="n"/>
+      <c r="I42" s="81" t="n"/>
+      <c r="J42" s="81" t="n"/>
+      <c r="K42" s="82" t="n"/>
+      <c r="L42" s="82" t="n"/>
+      <c r="M42" s="82" t="n"/>
+      <c r="N42" s="82" t="n"/>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>RealPage</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
         <is>
           <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
@@ -7072,7 +7186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H34"/>
+  <dimension ref="B2:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -7698,84 +7812,92 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="83" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="43" t="inlineStr">
+        <is>
+          <t>The Judy (Maple Grove &amp; Overland)</t>
+        </is>
+      </c>
+      <c r="C25" s="84" t="inlineStr">
+        <is>
+          <t>162</t>
+        </is>
+      </c>
+      <c r="D25" s="84" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E25" s="43" t="inlineStr">
+        <is>
+          <t>proposed - equity raise underway; construction targeted Q3 2026</t>
+        </is>
+      </c>
+      <c r="F25" s="43" t="n"/>
+      <c r="G25" s="43" t="inlineStr">
+        <is>
+          <t>Hawkins Companies OM (July 2026, research/oms/): 162-unit Class A garden (75x1BR $1,615 / 60x2BR / 27x3BR, avg $1,787 at 908sf) on 6.13 ac at 1770 S Maple Grove Rd, Boise — 3.4 mi from subject, inside the 5-mi ring. $41.7M TPC, GMP contract, construction targeted Q3 2026; OM lease-up: first occupancy month ~18 (=&gt; ~Q1 2028 first units), 20 units/mo absorption, ~42% occupied Yr 2. NOT tracked by CoStar or RealPage. Land-use analysis site 177: parcel S1124223215 in the developable-vacant set but zoned R-2 (Medium MF-threat, conditional) with 'single-family oriented' FLU — the OM proves the conditional path being exercised; reclassify from latent to tracked pipeline.</t>
+        </is>
+      </c>
+      <c r="H25" s="43" t="inlineStr">
+        <is>
+          <t>Hawkins Capital Markets OM — research/oms/Maple_Grove_Overland_Equity_Hawkins_OM.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="83" t="inlineStr">
         <is>
           <t>SHADOW SUPPLY (latent / untracked — watch list)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="50" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="50" t="inlineStr">
         <is>
           <t>Property / Site</t>
         </is>
       </c>
-      <c r="C27" s="50" t="inlineStr">
+      <c r="C28" s="50" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="D27" s="50" t="inlineStr">
+      <c r="D28" s="50" t="inlineStr">
         <is>
           <t>Est. Delivery</t>
         </is>
       </c>
-      <c r="E27" s="50" t="inlineStr">
+      <c r="E28" s="50" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F27" s="50" t="inlineStr">
+      <c r="F28" s="50" t="inlineStr">
         <is>
           <t>Leasing Pace</t>
         </is>
       </c>
-      <c r="G27" s="50" t="inlineStr">
+      <c r="G28" s="50" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H27" s="50" t="inlineStr">
+      <c r="H28" s="50" t="inlineStr">
         <is>
           <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="43" t="inlineStr">
-        <is>
-          <t>Emblem Meridian (Quarterra) / Artisan Victory Market site</t>
-        </is>
-      </c>
-      <c r="C28" s="84" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
-      </c>
-      <c r="D28" s="84" t="n"/>
-      <c r="E28" s="43" t="n"/>
-      <c r="F28" s="43" t="n"/>
-      <c r="G28" s="43" t="inlineStr">
-        <is>
-          <t>Land-use analysis site SM-76: ~12-ac BPS Eagle Road LLC assemblage on S Eagle Rd. 'Artisan Victory Market' (H-2022-0066) approved 2023 for 131 build-to-rent units + commercial but never built; superseded by Quarterra's 'Emblem Meridian' ~250-unit concept (pre-application June 2026). Closest large latent MF site to the subject (~1 mi).</t>
-        </is>
-      </c>
-      <c r="H28" s="43" t="inlineStr">
-        <is>
-          <t>https://boisedev.com/news/2026/06/10/meridian-emblem-victory-eagle-homes-apartment/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="43" t="inlineStr">
         <is>
-          <t>Tanner Creek apartments (Waltman/Johnson Ln)</t>
+          <t>Emblem Meridian (Quarterra) / Artisan Victory Market site</t>
         </is>
       </c>
       <c r="C29" s="84" t="inlineStr">
         <is>
-          <t>280</t>
+          <t>250</t>
         </is>
       </c>
       <c r="D29" s="84" t="n"/>
@@ -7783,24 +7905,24 @@
       <c r="F29" s="43" t="n"/>
       <c r="G29" s="43" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-15: Tanner Creek (heard Nov 2023; moved forward) — 83 SF homes + 45 townhomes + 280 phased apartments on ~38 ac, paired with ~30-ac Hawkins commercial between I-84 and Waltman Ln. Residential now being built by CBH Homes; the 280-unit apartment component is latent supply not yet in the CoStar/RealPage pipeline.</t>
+          <t>Land-use analysis site SM-76: ~12-ac BPS Eagle Road LLC assemblage on S Eagle Rd. 'Artisan Victory Market' (H-2022-0066) approved 2023 for 131 build-to-rent units + commercial but never built; superseded by Quarterra's 'Emblem Meridian' ~250-unit concept (pre-application June 2026). Closest large latent MF site to the subject (~1 mi).</t>
         </is>
       </c>
       <c r="H29" s="43" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2023/11/28/plans-for-two-large-developments-off-i-84-and-meridian-rd-move-forward/</t>
+          <t>https://boisedev.com/news/2026/06/10/meridian-emblem-victory-eagle-homes-apartment/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="43" t="inlineStr">
         <is>
-          <t>Graycliff Estates R-40 block</t>
+          <t>Tanner Creek apartments (Waltman/Johnson Ln)</t>
         </is>
       </c>
       <c r="C30" s="84" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>280</t>
         </is>
       </c>
       <c r="D30" s="84" t="n"/>
@@ -7808,40 +7930,44 @@
       <c r="F30" s="43" t="n"/>
       <c r="G30" s="43" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-3: Graycliff Estates (Star Development) approved preliminary plat of ~200 SF homes PLUS 224 apartments (R-40 high-density block) on ~52 ac; SF portion building since 2021. The 224-unit apartment block remains unbuilt latent supply.</t>
+          <t>Land-use analysis site SM-15: Tanner Creek (heard Nov 2023; moved forward) — 83 SF homes + 45 townhomes + 280 phased apartments on ~38 ac, paired with ~30-ac Hawkins commercial between I-84 and Waltman Ln. Residential now being built by CBH Homes; the 280-unit apartment component is latent supply not yet in the CoStar/RealPage pipeline.</t>
         </is>
       </c>
       <c r="H30" s="43" t="inlineStr">
         <is>
-          <t>https://www.weknowboise.com/graycliff-estates.php</t>
+          <t>https://boisedev.com/news/2023/11/28/plans-for-two-large-developments-off-i-84-and-meridian-rd-move-forward/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="43" t="inlineStr">
         <is>
-          <t>Touchmark Meadow Lake Village expansion</t>
-        </is>
-      </c>
-      <c r="C31" s="84" t="n"/>
+          <t>Graycliff Estates R-40 block</t>
+        </is>
+      </c>
+      <c r="C31" s="84" t="inlineStr">
+        <is>
+          <t>224</t>
+        </is>
+      </c>
       <c r="D31" s="84" t="n"/>
       <c r="E31" s="43" t="n"/>
       <c r="F31" s="43" t="n"/>
       <c r="G31" s="43" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-9: ~64 undeveloped ac of Touchmark's ~121-ac senior community. July 2025 development-modification agreement + rezone + PUD in progress to a broader 'Touchmark Mixed Use' (mixed housing types). Senior-oriented, but adds rental housing capacity 1.5 mi from subject.</t>
+          <t>Land-use analysis site SM-3: Graycliff Estates (Star Development) approved preliminary plat of ~200 SF homes PLUS 224 apartments (R-40 high-density block) on ~52 ac; SF portion building since 2021. The 224-unit apartment block remains unbuilt latent supply.</t>
         </is>
       </c>
       <c r="H31" s="43" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2025/07/14/touchmark-meridian-meadowlake-mixed-use/</t>
+          <t>https://www.weknowboise.com/graycliff-estates.php</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="43" t="inlineStr">
         <is>
-          <t>Ten Mile Crossing residual HDR parcels</t>
+          <t>Touchmark Meadow Lake Village expansion</t>
         </is>
       </c>
       <c r="C32" s="84" t="n"/>
@@ -7850,19 +7976,19 @@
       <c r="F32" s="43" t="n"/>
       <c r="G32" s="43" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-4: residential portion (R-15/R-8) of Brighton's Ten Mile Crossing at SW Overland &amp; Ten Mile — partially built (Cortland South Meridian + CBH SF); remaining High-Density Residential parcels planned/dormant, including an 8.6-ac and a 14.4-ac R-15 vacant parcel (highest-interest sites in the land-use ranking). Note: South Ridge II (164u UC, tracked in the chart) is rising in this same corridor.</t>
+          <t>Land-use analysis site SM-9: ~64 undeveloped ac of Touchmark's ~121-ac senior community. July 2025 development-modification agreement + rezone + PUD in progress to a broader 'Touchmark Mixed Use' (mixed housing types). Senior-oriented, but adds rental housing capacity 1.5 mi from subject.</t>
         </is>
       </c>
       <c r="H32" s="43" t="inlineStr">
         <is>
-          <t>https://www.brighton.co/brighton-place/ten-mile-crossing/</t>
+          <t>https://boisedev.com/news/2025/07/14/touchmark-meridian-meadowlake-mixed-use/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="43" t="inlineStr">
         <is>
-          <t>Brighton Apex R-15 parcel (Lake Hazel)</t>
+          <t>Ten Mile Crossing residual HDR parcels</t>
         </is>
       </c>
       <c r="C33" s="84" t="n"/>
@@ -7871,19 +7997,19 @@
       <c r="F33" s="43" t="n"/>
       <c r="G33" s="43" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-61: 15.1-ac R-15 (med-high-density) parcel on E Lake Hazel Rd inside Brighton's approved Apex/Pinnacle master-plan footprint; adjacent phases actively building. Latent MF-capable ground in the fast-growing S Meridian corridor.</t>
+          <t>Land-use analysis site SM-4: residential portion (R-15/R-8) of Brighton's Ten Mile Crossing at SW Overland &amp; Ten Mile — partially built (Cortland South Meridian + CBH SF); remaining High-Density Residential parcels planned/dormant, including an 8.6-ac and a 14.4-ac R-15 vacant parcel (highest-interest sites in the land-use ranking). Note: South Ridge II (164u UC, tracked in the chart) is rising in this same corridor.</t>
         </is>
       </c>
       <c r="H33" s="43" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2024/12/20/brighton-pinnacle-costco-meridian/</t>
+          <t>https://www.brighton.co/brighton-place/ten-mile-crossing/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="43" t="inlineStr">
         <is>
-          <t>Outer Banks Subdivision (TM Creek / Cobalt Dr)</t>
+          <t>Brighton Apex R-15 parcel (Lake Hazel)</t>
         </is>
       </c>
       <c r="C34" s="84" t="n"/>
@@ -7892,10 +8018,31 @@
       <c r="F34" s="43" t="n"/>
       <c r="G34" s="43" t="inlineStr">
         <is>
+          <t>Land-use analysis site SM-61: 15.1-ac R-15 (med-high-density) parcel on E Lake Hazel Rd inside Brighton's approved Apex/Pinnacle master-plan footprint; adjacent phases actively building. Latent MF-capable ground in the fast-growing S Meridian corridor.</t>
+        </is>
+      </c>
+      <c r="H34" s="43" t="inlineStr">
+        <is>
+          <t>https://boisedev.com/news/2024/12/20/brighton-pinnacle-costco-meridian/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="43" t="inlineStr">
+        <is>
+          <t>Outer Banks Subdivision (TM Creek / Cobalt Dr)</t>
+        </is>
+      </c>
+      <c r="C35" s="84" t="n"/>
+      <c r="D35" s="84" t="n"/>
+      <c r="E35" s="43" t="n"/>
+      <c r="F35" s="43" t="n"/>
+      <c r="G35" s="43" t="inlineStr">
+        <is>
           <t>Land-use analysis site SM-1: Ten Mile/I-84 high-density employment/mixed-use core (TMISAP) with heavy MF already delivered (Flats/Lofts/Cortland at Ten Mile). Outer Banks Subdivision approved 2021; balance of the ~198-ac district planned — further MF phases likely alongside the tracked pipeline.</t>
         </is>
       </c>
-      <c r="H34" s="43" t="inlineStr">
+      <c r="H35" s="43" t="inlineStr">
         <is>
           <t>https://boisedev.com/news/2021/12/17/outer-banks-pera-place/</t>
         </is>
@@ -7904,7 +8051,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B26:H26"/>
+    <mergeCell ref="B27:H27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>